<commit_message>
feat(shed): improve UX with wall separation, clickable parts, and 3D fixes
- Split Side Walls step into separate Left Wall and Right Wall steps (now 11 steps total)
- Make part IDs in Materials Needed section clickable to open part modal
- Add Excel download button for full parts list
- Remove T&G references from OSB flooring throughout (data, diagrams, Excel)
- Fix 3D rendering: cache materials for shingle swap, adjust camera lookAt, add shadows
- Update SVG diagrams to show wall build progression
</commit_message>
<xml_diff>
--- a/shed/data/shed_cut_sheet.xlsx
+++ b/shed/data/shed_cut_sheet.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cut Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cut Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,7 +59,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -73,11 +73,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -94,6 +122,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,6 +514,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -522,11 +553,11 @@
           <t>FOUNDATION</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -618,17 +649,18 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>FLOOR FRAME (Pressure Treated)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -728,7 +760,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>3/4" OSB T&amp;G</t>
+          <t>3/4" OSB</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -750,17 +782,18 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>WALL FRAMING (SPF or Similar)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -972,6 +1005,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
@@ -1058,6 +1092,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
@@ -1144,17 +1179,18 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>ROOF FRAMING</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1366,17 +1402,18 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>SIDING - LP SmartSide Cedar Texture Panel</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -1468,17 +1505,18 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
           <t>ROOF SHEATHING</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -1510,17 +1548,18 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ROOFING MATERIALS</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -1612,17 +1651,18 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
           <t>DOOR</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="5" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="5" t="n"/>
-      <c r="F55" s="5" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -1714,17 +1754,18 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
           <t>HARDWARE &amp; FASTENERS</t>
         </is>
       </c>
-      <c r="B60" s="5" t="n"/>
-      <c r="C60" s="5" t="n"/>
-      <c r="D60" s="5" t="n"/>
-      <c r="E60" s="5" t="n"/>
-      <c r="F60" s="5" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="n"/>
+      <c r="D60" s="8" t="n"/>
+      <c r="E60" s="8" t="n"/>
+      <c r="F60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -1966,17 +2007,19 @@
         </is>
       </c>
     </row>
+    <row r="69"/>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
           <t>MATERIALS PURCHASE SUMMARY</t>
         </is>
       </c>
-      <c r="B71" s="5" t="n"/>
-      <c r="C71" s="5" t="n"/>
-      <c r="D71" s="5" t="n"/>
-      <c r="E71" s="5" t="n"/>
-      <c r="F71" s="5" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="8" t="n"/>
+      <c r="D71" s="8" t="n"/>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -2376,7 +2419,7 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>3/4" T&amp;G</t>
+          <t>3/4"</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -2458,6 +2501,8 @@
         </is>
       </c>
     </row>
+    <row r="88"/>
+    <row r="89"/>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
@@ -2514,9 +2559,7 @@
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-    </row>
+    <row r="98"/>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
         <is>
@@ -2552,9 +2595,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr"/>
-    </row>
+    <row r="104"/>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>

</xml_diff>